<commit_message>
docs(order-management): lock 24.9 scope after per-item gate — per-installment refund primitive, amount-aware webhook in scope, paid_amount stays gross
</commit_message>
<xml_diff>
--- a/order_management/24.9-refund-management/24.9 - Refund Management.xlsx
+++ b/order_management/24.9-refund-management/24.9 - Refund Management.xlsx
@@ -24,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,8 +43,12 @@
       <color rgb="000563C1"/>
       <u val="single"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -86,8 +90,13 @@
         <fgColor rgb="00BFBFBF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E78"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -109,11 +118,25 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -158,6 +181,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -574,7 +606,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>8 requirement(s) to implement here (filter Build Focus = 'Implement here'). 0 covered elsewhere, 1 out of scope.</t>
+          <t>Scope locked 2026-07-03 (Step-1 gate complete — every verdict + 3 design decisions confirmed per-item). 8 requirement(s) to implement here, 0 covered elsewhere, 1 out of scope.</t>
         </is>
       </c>
     </row>
@@ -596,7 +628,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Story 24.9 asks for an admin Refund screen under Order Management that issues either a Manual (offline) refund or a Stripe refund against an order's payment plan, capped at the amount paid, with a mandatory reason, reflecting Stripe success/failure states. Re-verification against code confirms the read-side primitives are all BUILT and populated: Order.paid_amount is a running sum bumped by the Stripe webhook (cap is enforceable), PaymentTransaction.amount records per-installment paid amounts, Order/PaymentTransaction.stripe_charge_id identify Stripe-paid orders, the Stripe SDK is wired in external-api-service, OrderStatus.refunded/PaymentTransactionStatus.refunded exist, and an inbound charge.refunded webhook (handleChargeRefunded) already flips a PaymentTransaction to refunded and voids its invoice. The entire OM/refund module is net-new (no order module anywhere), and so are the Refund record model, the refund_failed enum value, and the outbound stripe.refunds.create wrapper — but all of these are story-owned net-new work built on top of working primitives, so they are Deliverable. The single genuine external gap is the absence of any write-path that records offline (check/wire/cash) payments as paid, which leaves only the Stripe-paid half of the method-availability requirement deliverable. Overall: largely Deliverable as a net-new module; 24.9-f is Partial pending an offline-payment-recording story, and the QuickBooks refund sync (24.9-i) is Out of Scope.</t>
+          <t>Admin refunds under OM: per-installment primitive + order-level composition (D1), net-new Refund ledger + refund_failed in PaymentTransactionStatus, stripe.refunds.create wrapper (single charge/call), amount-aware charge.refunded handler pulled into scope (D2), paid_amount stays gross (D3). 7 Deliverable, 24.9-f Partial (manual half gated on 24.8-&gt;24.7), 24.9-i Out of Scope (QB epic 65, un-ticketed; no refund story there — BA flagged).</t>
         </is>
       </c>
     </row>
@@ -672,7 +704,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Not started — analysis only</t>
+          <t>Not started — scope locked 2026-07-03 (gate complete)</t>
         </is>
       </c>
     </row>
@@ -798,7 +830,7 @@
       </c>
       <c r="L1" s="9" t="inlineStr">
         <is>
-          <t>Impl Status (2026-07-01)</t>
+          <t>Impl Status (2026-07-03)</t>
         </is>
       </c>
     </row>
@@ -830,12 +862,12 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>No order/order-management module or controller exists in any repo (verified against codebase map and controller listing), so the refund endpoint and UI wiring are net-new for this story, as for every OM story. It builds directly on the existing, populated Order / PaymentTransaction primitives. Building the net-new admin controller/service/DTO is Deliverable.</t>
+          <t>CONFIRMED 2026-07-03. Admin orders module now SHIPPED on dev (24.1–24.4 + 24.14), so refund routes are ADDITIVE routes on the shipped module (cheaper than the original net-new-module premise). Zero refund controllers/routes in any repo. Route shape per D1: POST body targets payment_transaction_id, or omits it for the order-level composition.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/prisma/schema.prisma:1540 (Order model); admin-backend-api/prisma/schema.prisma:2056 (PaymentTransaction model); codebase_map.md:373 (no OM module exists); admin-backend-api/src/admin/ppl-order/ppl-order.controller.ts:30 (@Controller pattern for net-new admin controller)</t>
+          <t>admin src/admin/orders/orders.controller.ts:41 (@Controller('orders') live: GET / :50, GET :id/notes :94, PATCH :id/notes :131); admin prisma/schema.prisma:1541 (Order), :2073 (PaymentTransaction); grep RefundController|refunds.create = zero in all 5 repos</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -856,7 +888,7 @@
       </c>
       <c r="L2" s="14" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate locked 2026-07-03: Deliverable confirmed (reason updated to additive-routes).</t>
         </is>
       </c>
     </row>
@@ -888,12 +920,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Re-verified: every primitive needed is built. Order.stripe_charge_id / PaymentTransaction.stripe_charge_id are written (ch_xxx from the succeeded PI's latest_charge), the Stripe SDK is already initialized in external-api-service (stripe.service.ts exposes createCustomer/createPaymentIntent/createSubscription/findChargeIdForInvoice etc.), and an inbound charge.refunded webhook already exercises the refund-on-charge model. No outbound stripe.refunds.create exists yet, but that wrapper plus the admin caller are ordinary net-new code on top of a populated charge id — there is no unbuilt upstream or unwritten existing field, so this is Deliverable (upgraded from Partial: the missing call is the story's own deliverable, not a missing primitive).</t>
+          <t>CONFIRMED 2026-07-03. All primitives populated; missing stripe.refunds.create wrapper is the story's own deliverable (external-api internal route). Per D1 the wrapper takes ONE charge + amount per call (each PT has its own ch_xxx); order-level composition loops legs newest-first in the admin service. Wrapper stays DB-free — admin does all persistence.</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>external-api-service/src/modules/stripe/services/stripe.service.ts:1-413 (Stripe SDK wired; no refunds.create; ends at findChargeIdForInvoice/extractStripeId); external-api-service/src/modules/webhook/services/webhook.service.ts:2879 (handleChargeRefunded uses stripe_charge_id); admin-backend-api/prisma/schema.prisma:1566 (Order.stripe_charge_id 'for refunds'); admin-backend-api/prisma/schema.prisma:2066 (PaymentTransaction.stripe_charge_id written from succeeded PI)</t>
+          <t>admin schema.prisma:1567 (Order.stripe_charge_id 'ch_xxx for refunds'), :2083 (PT.stripe_charge_id from succeeded PI latest_charge); ext stripe.service.ts (SDK wired, findChargeIdForInvoice :416, no refunds.create — grep zero); inbound precedent ext webhook.service.ts:3038</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr"/>
@@ -914,7 +946,7 @@
       </c>
       <c r="L3" s="14" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate locked 2026-07-03: Deliverable confirmed; wrapper shape fixed by D1 (single charge per call).</t>
         </is>
       </c>
     </row>
@@ -946,12 +978,12 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Re-verified: the terminal status is fully representable — PaymentTransactionStatus.refunded and OrderStatus.refunded both exist and are already written by the inbound charge.refunded webhook (proven write-path precedent). 'Record the refund internally' (amount, reason, method, who, when) needs a net-new Refund model, but adding that model + a manual-refund service that sets status=refunded without calling Stripe is story-owned net-new work on populated Order/PaymentTransaction rows. No external dependency or unwritten existing field gates it, so Deliverable (upgraded from Partial; consistent with treating net-new persistence as Deliverable per 24.9-e).</t>
+          <t>CONFIRMED 2026-07-03. Terminal status representable in both enums with proven transactional writer precedent (webhook). 'Record internally' = net-new Refund ledger model (absent from all 5 schemas; Int PK, NOT NULL where backfillable). DECIDED 2026-07-03 (D1): per-installment refunds are the primitive (Refund row targets one PaymentTransaction; cap = PT.amount − its prior Refund rows; refund_failed added to PaymentTransactionStatus); order-level refund = composition fanning out over installments newest-first; OrderStatus.refunded derived when all settled PTs refunded. Manual refund flips PaymentTransactionStatus.refunded.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/prisma/schema.prisma:497 (PaymentTransactionStatus.refunded); admin-backend-api/prisma/schema.prisma:426 (OrderStatus.refunded); external-api-service/src/modules/webhook/services/webhook.service.ts:2893 (existing writer of refunded status — write-path precedent); grep 'model Refund' across all schemas =&gt; none found (net-new, story-owned)</t>
+          <t>admin schema.prisma:426 (OrderStatus.refunded), :497 (PaymentTransactionStatus.refunded); ext webhook.service.ts:3048-3060 (tx precedent: PT-&gt;refunded + invoice-&gt;void); grep 'model Refund' = zero</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -972,7 +1004,7 @@
       </c>
       <c r="L4" s="14" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate locked 2026-07-03: Deliverable confirmed; D1 recorded.</t>
         </is>
       </c>
     </row>
@@ -1004,12 +1036,12 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>The cap is enforceable today: Order.paid_amount is a running sum written by the Stripe webhook on each succeeded installment (verified at webhook.service.ts: newPaidAmount = order.paid_amount.add(txPt.amount)), and PaymentTransaction.amount records per-installment paid amounts. The net-new endpoint validates refundAmount &lt;= paid_amount (less prior refunds) and accepts full or partial amounts — pure validation on populated data.</t>
+          <t>CONFIRMED 2026-07-03. Cap per D1 = target PT.amount − its prior Refund rows; order-level composition cap = Σ per-PT caps. DECIDED 2026-07-03 (D3): Order.paid_amount stays GROSS (never decremented; consistent with all readers: admin balance_due, exhibitor deriveOrderPaymentStatus/total_paid, agreement renderer); net paid derives as paid_amount − Σ Refund rows. Decimal cap-math per the deriveBalanceDue pattern.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/prisma/schema.prisma:1573 (Order.paid_amount 'Running sum...bumped by webhook'); external-api-service/src/modules/webhook/services/webhook.service.ts:2089-2105 (webhook computes &amp; writes paid_amount); admin-backend-api/prisma/schema.prisma:2062 (PaymentTransaction.amount)</t>
+          <t>admin schema.prisma:1578 (Order.paid_amount running sum), :2079 (PT.amount); ext webhook.service.ts:2111-2125 (sole paid_amount bumper); admin orders.helpers.ts:33 (deriveBalanceDue); reader sweep 2026-07-03: no paid_amount decrementer anywhere</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1030,7 +1062,7 @@
       </c>
       <c r="L5" s="14" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate locked 2026-07-03: Deliverable confirmed; D1 cap unit + D3 gross semantics recorded.</t>
         </is>
       </c>
     </row>
@@ -1062,12 +1094,12 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Mandatory-reason validation is trivially buildable in the net-new refund DTO/service (reject when empty). The reason's persistence target is the net-new Refund record (ordinary net-new column), and there is a class-validator DTO precedent (RefundDTO) in the unrelated PPL-lead refund flow. No external dependency. The 'for QuickBooks tracking' downstream sync is tracked separately as 24.9-i.</t>
+          <t>CONFIRMED 2026-07-03. Required non-empty DTO string + NOT NULL reason column on the net-new Refund model (grep refund_reason = zero). Class-validator precedent exists; reason doubles as the audit note (AdminAuditService throws on blank note). QB sync of the captured reason tracked as 24.9-i.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/src/admin/ppl-service-provider-detail-view/dto/index.ts:310 (RefundDTO precedent — class-validator reason field); grep 'refund_reason' across all schemas/src =&gt; none found (net-new, story-owned)</t>
+          <t>admin ppl-service-provider-detail-view/dto/index.ts:313 (RefundDTO precedent); admin admin-audit.service.ts:30/:50 (record/recordMany, throws on blank note)</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -1088,7 +1120,7 @@
       </c>
       <c r="L6" s="14" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate locked 2026-07-03: Deliverable confirmed.</t>
         </is>
       </c>
     </row>
@@ -1120,17 +1152,17 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Stripe-paid detection is fully deliverable now (presence of stripe_charge_id / stripe_payment_intent_id on the Order/PaymentTransaction), so the 'offer both methods' branch is buildable. BUT the manual-only branch presumes offline-paid orders exist, and re-verification confirms NO write-path records an offline/check/wire/cash payment as paid: the only code that bumps Order.paid_amount above zero is the Stripe webhook (exhibitor payments.service.ts:201 and cart.service.ts:1247 only initialize paid_amount to 0), and PaymentTransaction always carries non-null stripe_customer_id/stripe_payment_method_id (Stripe-only installments). CartPaymentMethod (check/bank_wire_ach/paypal) exists only on the CartPaymentPlan schedule, which is explicitly display/validation-only and never charged. So the offline-paid data this branch must discriminate is not produced by any code.</t>
+          <t>CONFIRMED Partial 2026-07-03. Stripe-detection half ships now (Stripe offered iff stripe_charge_id on the target PT; Manual always offered). Manual-only half has NO data producer: sole paid_amount bumper is the Stripe webhook; admin has no payment write-path; every PT is Stripe-shaped (NOT-NULL stripe cols); CartPaymentMethod is display-only. NO REWORK AT UNBLOCK: manual-paid PTs carry no charge id -&gt; Manual-only branch. Re-check at the 24.8 gate if classification source changes.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/prisma/schema.prisma:1564-1566 (Order stripe ids); admin-backend-api/prisma/schema.prisma:2067-2069 (PaymentTransaction non-null stripe_payment_method_id/stripe_customer_id); admin-backend-api/prisma/schema.prisma:2752 (CartPaymentMethod); admin-backend-api/prisma/schema.prisma:2838 ('Persisted for validation/display only — no charging happens here'); exhibitor-backend-api/src/payments/services/payments.service.ts:201 &amp; cart.service.ts:1247 (paid_amount only set to 0); webhook is sole bumper</t>
+          <t>admin schema.prisma:1567, :2084-2085 (PT NOT-NULL stripe cols), :2801-2808 (CartPaymentMethod), :2910 ('no charging happens here'); exh payments.service.ts:201 &amp; cart.service.ts:1316 (paid_amount init 0); ext webhook.service.ts:2112-2123 (sole bumper)</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>A write-path that records offline/manual (check/wire/cash) payments as paid against an order</t>
+          <t>Offline/manual payment producer: 24.8 (SBE-1132) payment_type migration + NOT-NULL relaxation, then 24.7 (SBE-1131) manual lifecycle — both In Progress, Prantik Saha</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr"/>
@@ -1146,7 +1178,7 @@
       </c>
       <c r="L7" s="14" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate locked 2026-07-03: Partial confirmed; dependency owners cited (24.8 -&gt; 24.7).</t>
         </is>
       </c>
     </row>
@@ -1178,12 +1210,12 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Re-verified: 'Refunded' is representable (PaymentTransactionStatus.refunded / OrderStatus.refunded, both already written). 'Refund Failed' has NO enum value today, but adding a refund_failed member to the enum is story-owned net-new schema work, identical in kind to adding the Refund model. Failure is captured synchronously from the stripe.refunds.create result/exception built in 24.9-b (the Stripe SDK returns refund.status and a refund.failed webhook event type is available in the SDK if async handling is wanted). No external dependency or unwritten existing field, so Deliverable (upgraded from Partial — the missing enum value is the story's own deliverable).</t>
+          <t>CONFIRMED 2026-07-03. refunded exists in both enums; refund_failed exists nowhere (grep zero) — story-owned enum addition into PaymentTransactionStatus per D1. Failure captured synchronously from wrapper result. SAME-SPRINT RIDER: extend exhibitor SETTLED_TRANSACTION_STATUSES one line, else refund-failed installments render payable. DECIDED 2026-07-03 (D2): amount-blind charge.refunded handler made amount-aware INSIDE SBE-1133 (external-api): full refund -&gt; flip PT + void invoice (as today); partial -&gt; PT status untouched, Refund ledger carries accounting; specs extended. Verified: no partial-refund logic and no refund issuer exists anywhere today (dashboard-only). Verified: worker charge/retry crons select only scheduled/failed — refunded/refund_failed PTs can never be re-charged.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/prisma/schema.prisma:491-500 (PaymentTransactionStatus: scheduled/processing/succeeded/failed/canceled/refunded — no refund_failed); admin-backend-api/prisma/schema.prisma:421-430 (OrderStatus — no refund_failed); external-api-service/src/modules/webhook/controllers/webhook.controller.ts:186 (charge.refunded already routed; refund.failed addable); grep 'refund_failed' =&gt; none found (net-new)</t>
+          <t>admin schema.prisma:491-501 (PaymentTransactionStatus, no refund_failed), :421-430 (OrderStatus); ext webhook.controller.ts:186-188; ext webhook.service.ts:3038-3060 (handler reads only charge.id — amount-blind, confirmed); exh orders.helpers.ts:31 (SETTLED set); worker payment-charge.service.ts:62-78</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr"/>
@@ -1204,7 +1236,7 @@
       </c>
       <c r="L8" s="14" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate locked 2026-07-03: Deliverable confirmed; D1 enum target + D2 handler change recorded.</t>
         </is>
       </c>
     </row>
@@ -1236,12 +1268,12 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Re-verified: all three enforcement pieces sit on story-owned or already-built primitives. Cap enforcement uses the populated Order.paid_amount (24.9-d). Mandatory-reason rejection is net-new DTO validation (24.9-e). Status-transition enforcement (idempotent Refunded / Refund Failed) drives off the net-new Refund record (24.9-c) and the net-new refund_failed enum value (24.9-g), both of which the story itself adds. There is no external/upstream blocker, so backend enforcement is Deliverable (upgraded from Partial).</t>
+          <t>CONFIRMED 2026-07-03. Cap = per-PT validation (D1); reason = DTO + NOT NULL column; transitions = status writes inside the same $transaction as ledger insert + wrapper call (webhook precedent). Residual one-liners: seed orders.refund after the orders.list block + @Permissions() per route; AdminAuditService.record/recordMany in-tx with the reason as note.</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/prisma/schema.prisma:1573 (paid_amount for caps); admin-backend-api/prisma/schema.prisma:491-500 (status enum, refund_failed to be added by this story); external-api-service/src/modules/webhook/services/webhook.service.ts:2893 (existing transactional status-write precedent)</t>
+          <t>admin permission.seeder.ts:1232 (orders block); admin admin-audit.service.ts:50 (tx-aware recordMany, 'order' in AdminAuditEntityType); ext webhook.service.ts:3048-3060 (transactional write precedent)</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr"/>
@@ -1262,7 +1294,7 @@
       </c>
       <c r="L9" s="14" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate locked 2026-07-03: Deliverable confirmed.</t>
         </is>
       </c>
     </row>
@@ -1294,17 +1326,17 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Capturing the reason is in scope (24.9-e), but the actual QuickBooks sync of refunds belongs to the accounting/integration epic, not this story. Re-verified: there is NO QuickBooks integration code anywhere — only dormant quickbooks_* columns and a QuickBooksSyncStatus enum with no writer. Pushing refunds to QuickBooks is out of this story's deliverable.</t>
+          <t>CONFIRMED Out of Scope 2026-07-03 (consistent with QB rows in 24.6/24.8). Reason capture in scope (24.9-e); QB sync not commissioned. Zero QB integration code in all 5 repos. QB home identified: epic 65 'Quickbooks Integration/Invoice Creation Process' on Admin Panel Page 2 (stories 65.1–65.5; NOT in Jira). BA FLAG: epic 65 has no refund/credit-memo story — 24.9's reason + Refund ledger are what that future sync consumes.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/prisma/schema.prisma:1567-1569 (quickbooks_order_id / quickbooks_sync_status columns, dormant); admin-backend-api/prisma/schema.prisma:474-481 (QuickBooksSyncStatus enum); codebase_map.md:378 ('QuickBooks: only dormant columns, NO integration code')</t>
+          <t>admin schema.prisma:1568-1570 (dormant quickbooks_* cols; Invoice :1988-1990), :474-481 (QuickBooksSyncStatus, writer-less); Jira search 'QuickBooks' = zero issues</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>QuickBooks integration (no write-path exists)</t>
+          <t>QuickBooks integration — Admin Panel Page 2, search 'Quickbooks Integration/Invoice Creation Process' (epic 65, un-ticketed)</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr"/>
@@ -1320,7 +1352,7 @@
       </c>
       <c r="L10" s="14" t="inlineStr">
         <is>
-          <t>Out of Scope — QuickBooks integration (no write-path exists)</t>
+          <t>Gate locked 2026-07-03: Out of Scope confirmed with epic-65 citation + BA gap flag.</t>
         </is>
       </c>
     </row>
@@ -1347,7 +1379,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1397,7 +1429,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Return available refund methods (always Manual; Stripe only when a stripe_charge_id exists) and the refundable cap (paid_amount minus prior refunds).</t>
+          <t>Per-installment refund eligibility: for each settled PT — method availability (always Manual; Stripe iff stripe_charge_id present) and remaining cap (PT.amount − Σ prior Refund rows); plus the order-level aggregate cap.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -1420,7 +1452,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Issue a Manual or Stripe refund for the order's payment plan: validate cap + mandatory reason, persist a Refund record, set status to Refunded or Refund Failed.</t>
+          <t>Issue a Manual or Stripe refund. Body: payment_transaction_id (per-installment primitive; omitted =&gt; order-level composition fanning out newest-first), amount, mandatory reason, send_notification (default true — 24.11 rider). Persists Refund ledger row(s), flips PaymentTransactionStatus to refunded/refund_failed, derives OrderStatus.refunded when all settled PTs refunded, audits in-tx.</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -1430,7 +1462,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>24.6 (Order Details refund action), 24.11 (refund email notice) — this story owns the canonical refunds endpoint.</t>
+          <t>24.6 (Order Details refund action), 24.10-f (cancel-with-refund composition), 24.11 (refund email toggle) — this story owns the canonical refunds endpoint.</t>
         </is>
       </c>
     </row>
@@ -1447,7 +1479,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>stripe.refunds.create wrapper against the order's stripe_charge_id, returning the Stripe refund result/status.</t>
+          <t>stripe.refunds.create wrapper: ONE charge + amount per call, DB-free, returns the Stripe refund result/status; admin composes multi-leg order-level refunds.</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -1457,7 +1489,34 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Internal external-api-service route called by the admin refunds service; not a public/admin route.</t>
+          <t>Reused by 24.10-f. Not a public/admin route.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>external-api-service: charge.refunded handler (scope change, D2)</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Make handleChargeRefunded amount-aware: full refund -&gt; flip PT + void invoice (as today); partial -&gt; leave PT status, Refund ledger carries accounting. Spec coverage extended.</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>24.9-g, 24.9-h</t>
+        </is>
+      </c>
+      <c r="E5" s="16" t="inlineStr">
+        <is>
+          <t>Same handler 24.10 copies PT-cancel patterns from — landing in 24.9 gives 24.10 a stable base.</t>
         </is>
       </c>
     </row>
@@ -1472,54 +1531,142 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="120" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="120" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B1" s="9" t="inlineStr">
-        <is>
-          <t>Open Question</t>
-        </is>
-      </c>
-      <c r="C1" s="9" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="D1" s="9" t="inlineStr">
-        <is>
-          <t>Resolution / Decision</t>
+      <c r="A1" s="17" t="inlineStr">
+        <is>
+          <t>Req</t>
+        </is>
+      </c>
+      <c r="B1" s="17" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="C1" s="17" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+      <c r="D1" s="17" t="inlineStr">
+        <is>
+          <t>Open Question / What is needed</t>
+        </is>
+      </c>
+      <c r="E1" s="17" t="inlineStr">
+        <is>
+          <t>Dependency (blocking story + Jira)</t>
+        </is>
+      </c>
+      <c r="F1" s="17" t="inlineStr">
+        <is>
+          <t>Assignee</t>
+        </is>
+      </c>
+      <c r="G1" s="17" t="inlineStr">
+        <is>
+          <t>Sprint / Jira status</t>
+        </is>
+      </c>
+      <c r="H1" s="17" t="inlineStr">
+        <is>
+          <t>Decision / Current direction</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Does 'payment plan' here mean the whole Order (cap = Order.paid_amount, status = OrderStatus.refunded) or an individual split installment (cap = PaymentTransaction.amount, status = PaymentTransactionStatus.refunded)? Both enums carry a `refunded` value and the inbound charge.refunded webhook operates per-PaymentTransaction, so the refund-cap and status-transition design differ for full-order vs per-installment refunds.</t>
-        </is>
-      </c>
-      <c r="C2" s="14" t="inlineStr">
-        <is>
-          <t>Open — for team discussion</t>
-        </is>
-      </c>
-      <c r="D2" s="14" t="inlineStr">
-        <is>
-          <t>Current direction (2026-07-01): — (pending). Leaning toward an order-level refund (cap = Order.paid_amount less prior refunds, status = OrderStatus.refunded) because the endpoint is order-scoped (/orders/:id/refunds) and the story refers to 'an order's payment plan' as a single unit; the per-PaymentTransaction charge.refunded precedent remains a viable alternative for split schedules. No code until the team confirms which unit the cap and status transition apply to.</t>
+      <c r="A2" s="16" t="inlineStr">
+        <is>
+          <t>24.9-f</t>
+        </is>
+      </c>
+      <c r="B2" s="16" t="inlineStr">
+        <is>
+          <t>Manual-only refund branch for offline-paid orders</t>
+        </is>
+      </c>
+      <c r="C2" s="16" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D2" s="16" t="inlineStr">
+        <is>
+          <t>A write-path that records offline/manual (check/wire/cash) payments as paid — no such data can exist today</t>
+        </is>
+      </c>
+      <c r="E2" s="16" t="inlineStr">
+        <is>
+          <t>24.8 (SBE-1132) payment_type migration + NOT-NULL relaxation -&gt; 24.7 (SBE-1131) manual lifecycle</t>
+        </is>
+      </c>
+      <c r="F2" s="16" t="inlineStr">
+        <is>
+          <t>Prantik Saha</t>
+        </is>
+      </c>
+      <c r="G2" s="16" t="inlineStr">
+        <is>
+          <t>Both In Progress</t>
+        </is>
+      </c>
+      <c r="H2" s="16" t="inlineStr">
+        <is>
+          <t>Stripe half ships with 24.9; manual half auto-works at unblock (charge-id-presence read needs no rework). Re-check at the 24.8 gate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="16" t="inlineStr">
+        <is>
+          <t>24.9-i</t>
+        </is>
+      </c>
+      <c r="B3" s="16" t="inlineStr">
+        <is>
+          <t>QuickBooks refund sync</t>
+        </is>
+      </c>
+      <c r="C3" s="16" t="inlineStr">
+        <is>
+          <t>Out of Scope</t>
+        </is>
+      </c>
+      <c r="D3" s="16" t="inlineStr">
+        <is>
+          <t>QB integration epic to consume the captured reason + Refund ledger</t>
+        </is>
+      </c>
+      <c r="E3" s="16" t="inlineStr">
+        <is>
+          <t>Epic 65, Admin Panel Page 2 (un-ticketed, no Jira issues exist)</t>
+        </is>
+      </c>
+      <c r="F3" s="16" t="inlineStr">
+        <is>
+          <t>— (BA)</t>
+        </is>
+      </c>
+      <c r="G3" s="16" t="inlineStr">
+        <is>
+          <t>Not commissioned</t>
+        </is>
+      </c>
+      <c r="H3" s="16" t="inlineStr">
+        <is>
+          <t>BA FLAG: epic 65 (65.1–65.5) covers invoices/payments only — no refund/credit-memo story exists anywhere.</t>
         </is>
       </c>
     </row>
@@ -1572,7 +1719,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Order Management (separate offline/manual payment-recording story — not yet built)</t>
+          <t>24.8 (SBE-1132) payment_type/payment_memo migration + NOT-NULL relaxation, then 24.7 (SBE-1131) manual Paid/Unpaid lifecycle — both In Progress, Prantik Saha</t>
         </is>
       </c>
     </row>
@@ -1589,7 +1736,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Accounting/QuickBooks integration epic</t>
+          <t>Epic 65 'Quickbooks Integration/Invoice Creation Process' — Admin Panel Page 2 (search the heading; stories 65.1–65.5; not in Jira). Epic 65 lacks a refund story — BA flagged.</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1751,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1624,86 +1771,158 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="14" t="inlineStr">
+      <c r="A2" s="18" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B2" s="16" t="inlineStr">
+        <is>
+          <t>Not started — Step-1 gate complete 2026-07-03; scope + 3 design decisions locked (D1 per-installment primitive / order-level composition; D2 amount-aware charge.refunded in scope; D3 paid_amount stays gross)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="18" t="inlineStr">
         <is>
           <t>Branch</t>
         </is>
       </c>
-      <c r="B2" s="14" t="inlineStr">
-        <is>
-          <t>— (not started). No SBE ticket / PR / Swagger tag yet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="B3" s="14" t="inlineStr">
-        <is>
-          <t>Not yet implemented — analysis/feasibility stage only. All 8 in-scope requirements are ◻ Not started.</t>
+      <c r="B3" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="14" t="inlineStr">
-        <is>
-          <t>Remaining — all in-scope</t>
-        </is>
-      </c>
-      <c r="B4" s="14" t="inlineStr">
-        <is>
-          <t>Unbuilt: 24.9-a, 24.9-b, 24.9-c, 24.9-d, 24.9-e, 24.9-f, 24.9-g, 24.9-h.</t>
+      <c r="A4" s="18" t="inlineStr">
+        <is>
+          <t>SBE ticket</t>
+        </is>
+      </c>
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>SBE-1133 (In Progress, Prantik Saha)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="14" t="inlineStr">
-        <is>
-          <t>Open decision — 'payment plan' scope</t>
-        </is>
-      </c>
-      <c r="B5" s="14" t="inlineStr">
-        <is>
-          <t>Whole Order (cap = Order.paid_amount, status = OrderStatus.refunded) vs individual split installment (cap = PaymentTransaction.amount, status = PaymentTransactionStatus.refunded). No code until answered.</t>
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>Commits</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="inlineStr">
-        <is>
-          <t>Dependency — offline payment write-path</t>
-        </is>
-      </c>
-      <c r="B6" s="14" t="inlineStr">
-        <is>
-          <t>Offline/manual (check/wire/cash) payment-recording write-path so manual-refund-only orders exist with a non-zero paid amount; gates the manual-only half of 24.9-f. Owner: separate OM story (not yet built).</t>
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="14" t="inlineStr">
-        <is>
-          <t>Dependency — QuickBooks</t>
-        </is>
-      </c>
-      <c r="B7" s="14" t="inlineStr">
-        <is>
-          <t>QuickBooks integration to sync issued refunds (no integration code exists; only dormant quickbooks_* columns and a writer-less QuickBooksSyncStatus enum); gates 24.9-i. Owner: Accounting/QuickBooks integration epic.</t>
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>Swagger tag</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="14" t="inlineStr">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>Build gates</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="18" t="inlineStr">
+        <is>
+          <t>Live smoke</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>Confirmed build scope</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>24.9-a/b/c/d/e/g/h + Stripe half of 24.9-f; incl. amount-aware charge.refunded handler (external-api) + exhibitor SETTLED extension rider</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>Remaining</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>All confirmed scope unbuilt</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="18" t="inlineStr">
+        <is>
+          <t>Not ready — see Open Questions</t>
+        </is>
+      </c>
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>24.9-f manual-only half; 24.9-i</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="18" t="inlineStr">
+        <is>
+          <t>External dependencies — see Cross-Epic Dependencies</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>Offline-payment producer (24.8 -&gt; 24.7); QuickBooks (epic 65, un-ticketed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="18" t="inlineStr">
         <is>
           <t>Out of API scope</t>
         </is>
       </c>
-      <c r="B8" s="14" t="inlineStr">
-        <is>
-          <t>Front-end refund-screen wiring; and 24.9-i (QuickBooks refund sync).</t>
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>Front-end refund-screen wiring</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(order-management): 24.9 Refund Management close-out — 24.9-f Partial -> Deliverable (post-merge)
Re-verified SBE-1133 against merged dev code. 24.9-f flipped Partial ->
Deliverable: its manual-only blocker dissolved because 24.7/24.8
(manual-payment lifecycle: payment_type NOT-NULL classifier, Stripe columns
nullable, markInstallmentPaid gross paid_amount bump) shipped on the same
feature/SBE-1125 branch and merged together. A manually-paid installment
carries no stripe_charge_id, so refund-options offers Manual-only and the
manual refund path executes. 24.9-i (QuickBooks) stays out of scope
(re-confirmed no QB writer in any repo). Counts now 8 Deliverable / 0 Partial
/ 1 OOS. Updated .md + .xlsx (Feasibility Counts, Requirements 24.9-f,
Open Questions, Cross-Epic Dependencies, Implementation Status).
</commit_message>
<xml_diff>
--- a/order_management/24.9-refund-management/24.9 - Refund Management.xlsx
+++ b/order_management/24.9-refund-management/24.9 - Refund Management.xlsx
@@ -652,8 +652,10 @@
           <t>Deliverable</t>
         </is>
       </c>
-      <c r="B9" s="4" t="n">
-        <v>7</v>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -662,8 +664,10 @@
           <t>Partial</t>
         </is>
       </c>
-      <c r="B10" s="5" t="n">
-        <v>1</v>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -704,7 +708,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Delivered — merged to dev 2026-07-05 (Phase 1 of the OM Phase-1 one-release).</t>
+          <t>Delivered — merged to dev 2026-07-05 (Phase 1). Post-merge re-verification 2026-07-06: 24.9-f flipped Partial → Deliverable (its manual-only blocker dissolved because 24.7/24.8 manual-payment lifecycle shipped on the SAME feature/SBE-1125 branch). Now 24.9-a..h all Deliverable &amp; shipped; only 24.9-i (QuickBooks) out of scope.</t>
         </is>
       </c>
     </row>
@@ -1137,7 +1141,7 @@
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Deliverable</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -1152,20 +1156,24 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>CONFIRMED Partial 2026-07-03. Stripe-detection half ships now (Stripe offered iff stripe_charge_id on the target PT; Manual always offered). Manual-only half has NO data producer: sole paid_amount bumper is the Stripe webhook; admin has no payment write-path; every PT is Stripe-shaped (NOT-NULL stripe cols); CartPaymentMethod is display-only. NO REWORK AT UNBLOCK: manual-paid PTs carry no charge id -&gt; Manual-only branch. Re-check at the 24.8 gate if classification source changes.</t>
+          <t>Gate-time verdict Partial (2026-07-03) → DELIVERABLE post-merge (re-verified 2026-07-06). Both halves live in the release: (Stripe half) refund-options offers Stripe iff the target PT has a stripe_charge_id, else Manual only; (manual-only half) the 'no offline-payment producer' blocker dissolved — 24.7/24.8 shipped on the same feature/SBE-1125 branch: payment_type is now a NOT-NULL classifier + Stripe columns nullable (24.8), and markInstallmentPaid records a manual (non-credit_card) installment paid + bumps paid_amount (24.8-c). A manually-paid PT carries no charge id → Manual-only branch; planLegs requires a charge id only for the Stripe method, so the manual refund executes. No rework needed.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>admin schema.prisma:1567, :2084-2085 (PT NOT-NULL stripe cols), :2801-2808 (CartPaymentMethod), :2910 ('no charging happens here'); exh payments.service.ts:201 &amp; cart.service.ts:1316 (paid_amount init 0); ext webhook.service.ts:2112-2123 (sole bumper)</t>
+          <t>admin schema.prisma: PaymentTransaction payment_type NOT-NULL + stripe_charge_id/stripe_payment_method_id/stripe_customer_id nullable ('NULL = manual non-card installment', story 24.8); order-payment-plan.service.ts:466 (markInstallmentPaid, gross paid_amount bump, 24.8-c); order-refund.service.ts:717 (Stripe method requires charge id), :851-853 (method availability)</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Offline/manual payment producer: 24.8 (SBE-1132) payment_type migration + NOT-NULL relaxation, then 24.7 (SBE-1131) manual lifecycle — both In Progress, Prantik Saha</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr"/>
+          <t>RESOLVED in-release — offline/manual payment producer landed via 24.8 (SBE-1132) + 24.7 (SBE-1131) on the same branch</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>[C3 build-once-reuse] OWNER — build here; manual-only branch unblocked in-release by 24.7/24.8</t>
+        </is>
+      </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
           <t>This option shall appear only if the payment was originally made through Stripe. If payment was made via check, wire transfer, cash, or any offline or manual method, only Manual Refund shall be available.</t>
@@ -1178,7 +1186,7 @@
       </c>
       <c r="L7" s="16" t="inlineStr">
         <is>
-          <t>Gate locked 2026-07-03: Partial confirmed; dependency owners cited (24.8 -&gt; 24.7). -&gt; ⚠️ Stripe-detection half DELIVERED (Stripe offered iff stripe_charge_id present; Manual always). Manual-only half still deferred — no offline-payment producer exists. Audit 2026-07-05 confirms partial-as-planned.</t>
+          <t>Post-merge 2026-07-06: Partial → ✅ DELIVERABLE (both halves). 24.7/24.8 producer shipped same release.</t>
         </is>
       </c>
     </row>
@@ -1599,17 +1607,17 @@
       </c>
       <c r="C2" s="16" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>RESOLVED → Deliverable (2026-07-06)</t>
         </is>
       </c>
       <c r="D2" s="16" t="inlineStr">
         <is>
-          <t>A write-path that records offline/manual (check/wire/cash) payments as paid — no such data can exist today</t>
+          <t>Was: a write-path recording offline/manual payments as paid. RESOLVED — the producer now exists in the same release (markInstallmentPaid, 24.8-c).</t>
         </is>
       </c>
       <c r="E2" s="16" t="inlineStr">
         <is>
-          <t>24.8 (SBE-1132) payment_type migration + NOT-NULL relaxation -&gt; 24.7 (SBE-1131) manual lifecycle</t>
+          <t>24.8 (SBE-1132) + 24.7 (SBE-1131) — shipped on the same feature/SBE-1125 branch</t>
         </is>
       </c>
       <c r="F2" s="16" t="inlineStr">
@@ -1619,12 +1627,12 @@
       </c>
       <c r="G2" s="16" t="inlineStr">
         <is>
-          <t>Both In Progress</t>
+          <t>Merged to dev</t>
         </is>
       </c>
       <c r="H2" s="16" t="inlineStr">
         <is>
-          <t>Stripe half ships with 24.9; manual half auto-works at unblock (charge-id-presence read needs no rework). Re-check at the 24.8 gate.</t>
+          <t>RESOLVED: markInstallmentPaid records manual installments paid; manually-paid PTs carry no charge id → Manual-only branch works exactly as designed. No rework was needed. Row retained for audit history.</t>
         </is>
       </c>
     </row>
@@ -1666,7 +1674,7 @@
       </c>
       <c r="H3" s="16" t="inlineStr">
         <is>
-          <t>BA FLAG: epic 65 (65.1–65.5) covers invoices/payments only — no refund/credit-memo story exists anywhere.</t>
+          <t>BA FLAG: epic 65 (65.1–65.5) covers invoices/payments only — no refund/credit-memo story exists anywhere. Re-confirmed 2026-07-06: no QB writer in any repo.</t>
         </is>
       </c>
     </row>
@@ -1709,7 +1717,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>A write-path that records offline/manual (check, wire, cash) payments as paid against an order (so manual-refund-only orders exist with a non-zero paid amount to refund against). Today only the Stripe webhook bumps Order.paid_amount.</t>
+          <t>[RESOLVED 2026-07-06] Write-path recording offline/manual (check, wire, cash) payments as paid — delivered in the same release by 24.8 (SBE-1132) + 24.7 (SBE-1131, markInstallmentPaid) on feature/SBE-1125. Stripe webhook no longer the sole paid_amount bumper.</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -1874,7 +1882,7 @@
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>24.9-a/b/c/d/e/g/h delivered + Stripe-detection half of 24.9-f. Refund ledger + refund_failed status; POST /orders/:id/refunds, GET /orders/:id/refund-options.</t>
+          <t>24.9-a/b/c/d/e/f/g/h delivered (24.9-f both halves — post-merge). Refund ledger + refund_failed status; POST /orders/:id/refunds, GET /orders/:id/refund-options.</t>
         </is>
       </c>
     </row>
@@ -1886,7 +1894,7 @@
       </c>
       <c r="B11" s="16" t="inlineStr">
         <is>
-          <t>24.9-f manual-only half still deferred (no offline-payment producer yet); 24.9-i (QuickBooks) out of scope.</t>
+          <t>Only 24.9-i (QuickBooks) out of scope. 24.9-f manual-only half now live (24.7/24.8 landed in the same release, 2026-07-06).</t>
         </is>
       </c>
     </row>
@@ -1898,7 +1906,7 @@
       </c>
       <c r="B12" s="16" t="inlineStr">
         <is>
-          <t>24.9-f manual-only half; 24.9-i</t>
+          <t>24.9-i (QuickBooks) only.</t>
         </is>
       </c>
     </row>
@@ -1910,7 +1918,7 @@
       </c>
       <c r="B13" s="16" t="inlineStr">
         <is>
-          <t>Offline-payment producer (24.8 -&gt; 24.7); QuickBooks (epic 65, un-ticketed)</t>
+          <t>Offline-payment producer dependency RESOLVED in-release (24.8 -&gt; 24.7 shipped on the same branch). QuickBooks (epic 65, un-ticketed) still open.</t>
         </is>
       </c>
     </row>

</xml_diff>